<commit_message>
Split Oracle's FY2032-onward principal by decade
The ladder's combined $90.25B bar is now shown by decade under it in the
app and as SUMIFS formulas beside the calendar on the workbook's Payment
dates sheet, with a check that the decades equal Thereafter.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/oracle_liquidity.xlsx
+++ b/samples/oracle_liquidity.xlsx
@@ -10373,6 +10373,12 @@
       <x:c r="D48" s="470" t="str">
         <x:v>Through</x:v>
       </x:c>
+      <x:c r="E48" s="469" t="str">
+        <x:v>FY2032 onward, by decade</x:v>
+      </x:c>
+      <x:c r="F48" s="470" t="str">
+        <x:v>Principal (USD millions)</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="18" customHeight="1">
       <x:c r="A49" s="378" t="str">
@@ -10388,6 +10394,13 @@
       <x:c r="D49" s="471" t="d">
         <x:v>2027-05-31T00:00:00.000Z</x:v>
       </x:c>
+      <x:c r="E49" s="378" t="str">
+        <x:v>FY2032–36</x:v>
+      </x:c>
+      <x:c r="F49" s="472" t="n">
+        <x:f>SUMIFS($E$95:$E$152,$B$95:$B$152,"&gt;="&amp;DATE(2031,6,1),$B$95:$B$152,"&lt;="&amp;DATE(2036,5,31),$F$95:$F$152,"&lt;&gt;Term loan")</x:f>
+        <x:v>26500000000</x:v>
+      </x:c>
     </x:row>
     <x:row r="50" ht="18" customHeight="1">
       <x:c r="A50" s="378" t="str">
@@ -10403,6 +10416,13 @@
       <x:c r="D50" s="471" t="d">
         <x:v>2028-05-31T00:00:00.000Z</x:v>
       </x:c>
+      <x:c r="E50" s="378" t="str">
+        <x:v>FY2037–46</x:v>
+      </x:c>
+      <x:c r="F50" s="472" t="n">
+        <x:f>SUMIFS($E$95:$E$152,$B$95:$B$152,"&gt;="&amp;DATE(2036,6,1),$B$95:$B$152,"&lt;="&amp;DATE(2046,5,31),$F$95:$F$152,"&lt;&gt;Term loan")</x:f>
+        <x:v>20750000000</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" ht="18" customHeight="1">
       <x:c r="A51" s="378" t="str">
@@ -10418,6 +10438,13 @@
       <x:c r="D51" s="471" t="d">
         <x:v>2029-05-31T00:00:00.000Z</x:v>
       </x:c>
+      <x:c r="E51" s="378" t="str">
+        <x:v>FY2047–56</x:v>
+      </x:c>
+      <x:c r="F51" s="472" t="n">
+        <x:f>SUMIFS($E$95:$E$152,$B$95:$B$152,"&gt;="&amp;DATE(2046,6,1),$B$95:$B$152,"&lt;="&amp;DATE(2056,5,31),$F$95:$F$152,"&lt;&gt;Term loan")</x:f>
+        <x:v>31000000000</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" ht="18" customHeight="1">
       <x:c r="A52" s="378" t="str">
@@ -10433,6 +10460,13 @@
       <x:c r="D52" s="471" t="d">
         <x:v>2030-05-31T00:00:00.000Z</x:v>
       </x:c>
+      <x:c r="E52" s="378" t="str">
+        <x:v>FY2057–66</x:v>
+      </x:c>
+      <x:c r="F52" s="472" t="n">
+        <x:f>SUMIFS($E$95:$E$152,$B$95:$B$152,"&gt;="&amp;DATE(2056,6,1),$B$95:$B$152,"&lt;="&amp;DATE(2066,5,31),$F$95:$F$152,"&lt;&gt;Term loan")</x:f>
+        <x:v>12000000000</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="18" customHeight="1">
       <x:c r="A53" s="378" t="str">
@@ -10448,6 +10482,13 @@
       <x:c r="D53" s="471" t="d">
         <x:v>2031-05-31T00:00:00.000Z</x:v>
       </x:c>
+      <x:c r="E53" s="473" t="str">
+        <x:v>Sum of decades</x:v>
+      </x:c>
+      <x:c r="F53" s="474" t="n">
+        <x:f>SUM(F49:F52)</x:f>
+        <x:v>90250000000</x:v>
+      </x:c>
     </x:row>
     <x:row r="54" ht="18" customHeight="1">
       <x:c r="A54" s="378" t="str">
@@ -10462,6 +10503,13 @@
       </x:c>
       <x:c r="D54" s="411" t="str">
         <x:v>Final maturity</x:v>
+      </x:c>
+      <x:c r="E54" s="378" t="str">
+        <x:v>Less Thereafter (C54); should be 0</x:v>
+      </x:c>
+      <x:c r="F54" s="472" t="n">
+        <x:f>F53-C54</x:f>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="18" customHeight="1">

</xml_diff>